<commit_message>
Re-verify time-sensitive test cases and add validity column
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LR7nyPU9eWbuGKSxbbvrSC
</commit_message>
<xml_diff>
--- a/testsets/gz_xpeng_nav_supplement.xlsx
+++ b/testsets/gz_xpeng_nav_supplement.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -439,7 +439,8 @@
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,6 +486,11 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>有效期至</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>需高德复核</t>
         </is>
       </c>
@@ -530,6 +536,11 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>是：确认正佳确无海底捞</t>
         </is>
       </c>
@@ -575,6 +586,11 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -620,6 +636,11 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>是：确认现址</t>
         </is>
       </c>
@@ -665,6 +686,11 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -710,6 +736,11 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -740,12 +771,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2024 年报道称引入啫火、猫员外、Manner、茉莉奶白、DQ</t>
+          <t>360地图有 POI「啫火(智慧城广百广场店)」，人均约78元；2024 年揭牌报道提到入驻</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>品牌可能已撤店：若撤店应兜底而不是硬导航</t>
+          <t>品牌门店可能变动：若撤店应兜底而不是硬导航</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -754,6 +785,11 @@
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>不定期复核</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>是：确认是否仍营业</t>
         </is>
@@ -780,12 +816,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>智慧城广百广场内 Manner（若仍营业）</t>
+          <t>Manner Coffee(智慧城广百广场店)，小餐车形式（若仍营业）</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>同上 2024 年报道</t>
+          <t>360地图有 POI，但 Manner 官网广州门店列表未见该店，可能已撤或改名</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -799,6 +835,11 @@
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>不定期复核</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>是：确认是否仍营业</t>
         </is>
@@ -845,6 +886,11 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
           <t>否</t>
         </is>
       </c>
@@ -890,6 +936,11 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>是：确认高德 POI 名</t>
         </is>
       </c>
@@ -935,6 +986,11 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>否</t>
         </is>
       </c>
@@ -980,6 +1036,11 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
           <t>是：确认旧址是否仍有门店</t>
         </is>
       </c>
@@ -1025,6 +1086,11 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>是：确认 T2北门 POI</t>
         </is>
       </c>
@@ -1070,6 +1136,11 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -1115,6 +1186,11 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
           <t>否</t>
         </is>
       </c>
@@ -1160,6 +1236,11 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -1205,6 +1286,11 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
           <t>否</t>
         </is>
       </c>
@@ -1250,6 +1336,11 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -1295,6 +1386,11 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -1320,12 +1416,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>广东奥林匹克体育中心体育场（2026-11-07/08）</t>
+          <t>广东奥林匹克体育中心体育场（2026-11-07/08，门票已售罄）</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>王力宏官网公告；本地宝演唱会排期</t>
+          <t>王力宏官网 2026-09-21 公告、10-16 更新售罄；新浪有“11-06 至 08 三场”说法，以官网为准</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1338,7 +1434,12 @@
           <t>高</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1366,7 +1467,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>新浪、广州日报下半年演唱会汇总</t>
+          <t>HK01、大河票务等多家报道一致</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1379,7 +1480,12 @@
           <t>高</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-06</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1407,7 +1513,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>演唱会汇总</t>
+          <t>文旅部演出审批公示（21财经、新浪报道）</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1420,7 +1526,12 @@
           <t>高</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-06</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1461,7 +1572,12 @@
           <t>高</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1489,7 +1605,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>演唱会汇总</t>
+          <t>广东发布（新浪财经 2026-09-22 转载），目前单一来源</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1502,7 +1618,12 @@
           <t>高</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1545,6 +1666,11 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
+          <t>2027-07（下届乞巧节公布前）</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -1588,7 +1714,12 @@
           <t>高</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1629,7 +1760,12 @@
           <t>中</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1652,12 +1788,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>华南植物园；资料为 07:30-17:30（较旧，需复核）</t>
+          <t>华南植物园；07:30-17:30（17:30 停止入园），温室时间另计</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>本地宝/大河票务（2022 年资料）</t>
+          <t>华南植物园官网、携程</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1670,7 +1806,12 @@
           <t>中</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1711,7 +1852,12 @@
           <t>中</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1752,7 +1898,12 @@
           <t>中</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1795,6 +1946,11 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
           <t>是：确认高德是否仍有 POI</t>
         </is>
       </c>
@@ -1840,6 +1996,11 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -1885,6 +2046,11 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
@@ -1928,7 +2094,12 @@
           <t>中</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1969,7 +2140,12 @@
           <t>低</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2012,6 +2188,11 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
           <t>是：逐个验证模型给的店名</t>
         </is>
       </c>
@@ -2055,7 +2236,12 @@
           <t>中</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2096,7 +2282,12 @@
           <t>低</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2137,7 +2328,12 @@
           <t>低</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2178,7 +2374,12 @@
           <t>低</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2219,7 +2420,12 @@
           <t>低</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2260,7 +2466,12 @@
           <t>低</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2296,7 +2507,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>时效性=高 的条目（演出、品牌门店、乞巧节）会过期，每次跑之前确认一遍。</t>
+          <t>时效性=高 的条目已于 2026-10-22 复核，均仍有效；“有效期至”过后需替换（演出类 12-20 后全部过期）。</t>
         </is>
       </c>
     </row>

</xml_diff>